<commit_message>
Billing pour play store,  fix bug, comment jouer, sharescreen, multifix
</commit_message>
<xml_diff>
--- a/backend/src/data/Onskoné_2405.xlsx
+++ b/backend/src/data/Onskoné_2405.xlsx
@@ -2229,10 +2229,10 @@
     <t>Generosity</t>
   </si>
   <si>
-    <t>Qu'est-ce que tu fais anonyment et généreusement, sans attendre de retour ?</t>
-  </si>
-  <si>
-    <t>What do you do anonymously and generously, expecting nothing in return?</t>
+    <t>Qu'est-ce que tu fais pour les autres sans le crier sur tous les toits ?</t>
+  </si>
+  <si>
+    <t>What do you do for others without shouting it from the rooftops?</t>
   </si>
   <si>
     <t>Quel geste d'amour que tu as reçu, qui t'a marqué récemment ?</t>
@@ -2457,10 +2457,10 @@
     <t>Mood</t>
   </si>
   <si>
-    <t>Comment décrirais-tu ton humeur actuelle en un mot ?</t>
-  </si>
-  <si>
-    <t>How would you describe your current mood in one word?</t>
+    <t>Comment décrirais-tu ton humeur actuelle en quelques mots ?</t>
+  </si>
+  <si>
+    <t>How would you describe your current mood in a few words?</t>
   </si>
   <si>
     <t>Dans ta vie actuelle, quelle est la chose que tu as idéalisée avant d'en faire l'expérience ?</t>
@@ -4617,10 +4617,10 @@
     <t>Mental Health</t>
   </si>
   <si>
-    <t>Décris ton état de santé mentale en un mot</t>
-  </si>
-  <si>
-    <t>Describe your mental health in one word.</t>
+    <t>Décris ton état de santé mentale en une phrase</t>
+  </si>
+  <si>
+    <t>Describe your mental health in one sentence.</t>
   </si>
   <si>
     <t>Quelle est ta scène de film préférée ?</t>

</xml_diff>